<commit_message>
torque paper text and figures updated
</commit_message>
<xml_diff>
--- a/Documentation/Reports and Papers/Knee_Torque_Test/Tables/PinnedFlexor_Preopt_GoF.xlsx
+++ b/Documentation/Reports and Papers/Knee_Torque_Test/Tables/PinnedFlexor_Preopt_GoF.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FlxPinPreGof" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preopt GoF" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -428,7 +428,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Hunt RMSE (N·m)</t>
+          <t>Hunt RMSE</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -438,22 +438,37 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Hunt Max (N·m)</t>
+          <t>Hunt Max</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Unopt RMSE (N·m)</t>
+          <t>Improved char alone RMSE</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Unopt FVU</t>
+          <t>Improved char alone FVU</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Unopt Max (N·m)</t>
+          <t>Improved char alone Max</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Back-calculated (hybrid) RMSE</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Back-calculated (hybrid) FVU</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Back-calculated (hybrid) Max</t>
         </is>
       </c>
     </row>
@@ -464,22 +479,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5.762</v>
+        <v>5.779</v>
       </c>
       <c r="C2" t="n">
-        <v>1.1693</v>
+        <v>1.1761</v>
       </c>
       <c r="D2" t="n">
-        <v>9.534000000000001</v>
+        <v>9.798</v>
       </c>
       <c r="E2" t="n">
-        <v>7.617</v>
+        <v>4.871</v>
       </c>
       <c r="F2" t="n">
-        <v>2.1278</v>
+        <v>0.8354</v>
       </c>
       <c r="G2" t="n">
-        <v>25.531</v>
+        <v>9.865</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.635</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.09909999999999999</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3.842</v>
       </c>
     </row>
     <row r="3">
@@ -489,22 +513,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.101</v>
+        <v>6.633</v>
       </c>
       <c r="C3" t="n">
-        <v>3.1245</v>
+        <v>3.2313</v>
       </c>
       <c r="D3" t="n">
-        <v>13.144</v>
+        <v>11.409</v>
       </c>
       <c r="E3" t="n">
-        <v>9.694000000000001</v>
+        <v>6.074</v>
       </c>
       <c r="F3" t="n">
-        <v>2.1149</v>
+        <v>2.709</v>
       </c>
       <c r="G3" t="n">
-        <v>21.076</v>
+        <v>9.262</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2.187</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.1184</v>
+      </c>
+      <c r="J3" t="n">
+        <v>4.243</v>
       </c>
     </row>
     <row r="4">
@@ -514,22 +547,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6.51</v>
+        <v>5.315</v>
       </c>
       <c r="C4" t="n">
-        <v>1.3069</v>
+        <v>0.9408</v>
       </c>
       <c r="D4" t="n">
-        <v>15.886</v>
+        <v>9.991</v>
       </c>
       <c r="E4" t="n">
-        <v>8.803000000000001</v>
+        <v>4.465</v>
       </c>
       <c r="F4" t="n">
-        <v>1.938</v>
+        <v>0.664</v>
       </c>
       <c r="G4" t="n">
-        <v>26.264</v>
+        <v>9.536</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.246</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.0409</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2.275</v>
       </c>
     </row>
     <row r="5">
@@ -539,22 +581,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.955</v>
+        <v>3.945</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6783</v>
+        <v>0.675</v>
       </c>
       <c r="D5" t="n">
-        <v>7.846</v>
+        <v>7.527</v>
       </c>
       <c r="E5" t="n">
-        <v>6.373</v>
+        <v>3.226</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5935</v>
+        <v>0.4512</v>
       </c>
       <c r="G5" t="n">
-        <v>16.859</v>
+        <v>7.376</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2.085</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.0755</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3.073</v>
       </c>
     </row>
     <row r="6">
@@ -564,22 +615,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6.432</v>
+        <v>6.206</v>
       </c>
       <c r="C6" t="n">
-        <v>2.1469</v>
+        <v>2.2037</v>
       </c>
       <c r="D6" t="n">
-        <v>11.339</v>
+        <v>10.604</v>
       </c>
       <c r="E6" t="n">
-        <v>8.656000000000001</v>
+        <v>5.472</v>
       </c>
       <c r="F6" t="n">
-        <v>2.1213</v>
+        <v>1.7722</v>
       </c>
       <c r="G6" t="n">
-        <v>23.303</v>
+        <v>9.563000000000001</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.911</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.1088</v>
+      </c>
+      <c r="J6" t="n">
+        <v>4.043</v>
       </c>
     </row>
     <row r="7">
@@ -589,22 +649,38 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5.232</v>
+        <v>4.63</v>
       </c>
       <c r="C7" t="n">
-        <v>0.9926</v>
+        <v>0.8079</v>
       </c>
       <c r="D7" t="n">
-        <v>11.866</v>
+        <v>8.759</v>
       </c>
       <c r="E7" t="n">
-        <v>7.588</v>
+        <v>3.845</v>
       </c>
       <c r="F7" t="n">
-        <v>1.2657</v>
+        <v>0.5576</v>
       </c>
       <c r="G7" t="n">
-        <v>21.562</v>
+        <v>8.456</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.666</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.0582</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2.674</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Basis: Hunt-equation and improved-characterization columns are scored head-to-head on the measured points where the Hunt prediction is defined (75/90, 17/20, 14/19, 15/22 points in panel order); the back-calculated (hybrid) column is scored on all measured points. Torque residuals in N*m. Matches tab:FlxPinPreGof, Main.tex 2026-10-19.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>